<commit_message>
Excel R3.2 con el .anl R3.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R3.2.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R3.2.xlsx
@@ -12444,7 +12444,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 19,691.90 kg (.anl R3.1, masa de contravientos en cabezas de columna).</t>
+          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 19,691.90 kg (.anl R3.2).</t>
         </is>
       </c>
       <c r="F60" s="4" t="s">
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="C73" s="16">
-        <v>2.788</v>
+        <v>2.787</v>
       </c>
       <c r="D73" s="16">
-        <v>2.29</v>
+        <v>2.289</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
@@ -14061,11 +14061,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.3076876409100227</v>
+        <v>1.3081568506842995</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.5920668746101059</v>
+        <v>1.5927624040441863</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14119,11 +14119,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$76</f>
-        <v>1.3076876409100227</v>
+        <v>1.3081568506842995</v>
       </c>
       <c r="D78" s="21">
         <f>$D$76</f>
-        <v>1.5920668746101059</v>
+        <v>1.5927624040441863</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14179,11 +14179,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.3076876409100227</v>
+        <v>1.3081568506842995</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.5920668746101059</v>
+        <v>1.5927624040441863</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="C92" s="13">
         <f>$C$73</f>
-        <v>2.788</v>
+        <v>2.787</v>
       </c>
       <c r="D92" s="53">
         <v>1.82038061</v>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.3076876409100227</v>
+        <v>1.3081568506842995</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="C101" s="13">
         <f>$D$73</f>
-        <v>2.29</v>
+        <v>2.289</v>
       </c>
       <c r="D101" s="53">
         <v>2.72429032</v>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.5920668746101059</v>
+        <v>1.5927624040441863</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14793,11 +14793,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$76</f>
-        <v>1.3076876409100227</v>
+        <v>1.3081568506842995</v>
       </c>
       <c r="D104" s="13">
         <f>$D$76</f>
-        <v>1.5920668746101059</v>
+        <v>1.5927624040441863</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14823,11 +14823,11 @@
       </c>
       <c r="C105" s="13">
         <f>-$C$76</f>
-        <v>-1.3076876409100227</v>
+        <v>-1.3081568506842995</v>
       </c>
       <c r="D105" s="13">
         <f>-$D$76</f>
-        <v>-1.5920668746101059</v>
+        <v>-1.5927624040441863</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14853,11 +14853,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.26901002898720466</v>
+        <v>0.26910655214077017</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.3275108999197932</v>
+        <v>0.32765398026051834</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>

</xml_diff>